<commit_message>
docs: finalizar entregables de pruebas y Scrum
</commit_message>
<xml_diff>
--- a/entregables/02-Historias-y-Casos-de-Prueba.xlsx
+++ b/entregables/02-Historias-y-Casos-de-Prueba.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias de usuario" sheetId="1" r:id="R0b22ef839aa24a11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de prueba" sheetId="2" r:id="Rab28863aee4d4f3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trazabilidad" sheetId="3" r:id="R4aaa6538491d4624"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablero Scrum" sheetId="4" r:id="R1fcc2f5288494fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias de usuario" sheetId="1" r:id="R62e8d70ec4dc41fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de prueba" sheetId="2" r:id="R86f13aaa46eb41dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trazabilidad" sheetId="3" r:id="R9a6c8faf3e7442fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablero Scrum" sheetId="4" r:id="R280d5880e5584652"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2133,7 +2133,7 @@
     <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="70" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="68" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -2153,13 +2153,13 @@
         <x:v>Prioridad</x:v>
       </x:c>
       <x:c r="F1" s="33" t="str">
-        <x:v>Fecha objetivo</x:v>
-      </x:c>
-      <x:c r="G1" s="33" t="str">
-        <x:v>Estado al 14/10 y criterio de aceptación</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="60" customHeight="1">
+        <x:v>Fecha / hito del cronograma</x:v>
+      </x:c>
+      <x:c r="G1" s="11" t="str">
+        <x:v>Criterio de aceptación y evidencia integrada</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A2" s="16" t="str">
         <x:v>SQA-01</x:v>
       </x:c>
@@ -2179,15 +2179,15 @@
         <x:v>14–18/10</x:v>
       </x:c>
       <x:c r="G2" s="16" t="str">
-        <x:v>En curso. Registrar objetivo, avance, siguiente paso y bloqueos de cada sesión realizada.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="60" customHeight="1">
+        <x:v>Backlog con 10 tareas, responsables, revisores y criterios de aceptación. El tablero de GitHub enlaza cada tarea con un Issue.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A3" s="16" t="str">
         <x:v>SQA-02</x:v>
       </x:c>
       <x:c r="B3" s="16" t="str">
-        <x:v>Confirmar Docker/MySQL y documentar ejecución en VS Code</x:v>
+        <x:v>Levantar y documentar Docker/MySQL y ejecución en VS Code</x:v>
       </x:c>
       <x:c r="C3" s="16" t="str">
         <x:v>Noemy Molina Garron</x:v>
@@ -2202,10 +2202,10 @@
         <x:v>14/10</x:v>
       </x:c>
       <x:c r="G3" s="16" t="str">
-        <x:v>Entorno levantado 12/10; revisar guía, comandos de inicio, comprobación, Cypress y apagado.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="60" customHeight="1">
+        <x:v>Entorno Docker/MySQL levantado el 12/10, según lo informado por el equipo; guía de VS Code incluye inicio, comprobación, ejecución y detención.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="16" t="str">
         <x:v>SQA-03</x:v>
       </x:c>
@@ -2225,10 +2225,10 @@
         <x:v>15/10</x:v>
       </x:c>
       <x:c r="G4" s="16" t="str">
-        <x:v>En curso. Plan coherente con CP-01, matriz y brechas reales.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="60" customHeight="1">
+        <x:v>Plan documenta alcance, CP-01 como smoke test, criterios de entrada/salida y riesgos de ejecución.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A5" s="16" t="str">
         <x:v>SQA-04</x:v>
       </x:c>
@@ -2248,10 +2248,10 @@
         <x:v>16/10</x:v>
       </x:c>
       <x:c r="G5" s="16" t="str">
-        <x:v>Pendiente. Cada caso tiene precondición, datos, pasos, resultado y trazabilidad.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="60" customHeight="1">
+        <x:v>CP-01 a CP-07 describen portada y flujos de administración con precondiciones, datos, pasos y resultados esperados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
         <x:v>SQA-05</x:v>
       </x:c>
@@ -2271,10 +2271,10 @@
         <x:v>16/10</x:v>
       </x:c>
       <x:c r="G6" s="16" t="str">
-        <x:v>En curso. Historias, criterios y pruebas concuerdan con la aplicación y spec.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="60" customHeight="1">
+        <x:v>HU-07 a HU-13 y CP-08 a CP-15 cubren registro, acceso, cita, consulta y cierre de sesión del paciente.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="16" t="str">
         <x:v>SQA-06</x:v>
       </x:c>
@@ -2294,10 +2294,10 @@
         <x:v>17/10</x:v>
       </x:c>
       <x:c r="G7" s="16" t="str">
-        <x:v>Pendiente. Login, dashboard, atención, perfil, contraseña y logout documentados.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="60" customHeight="1">
+        <x:v>CP-17 a CP-21 cubren login, dashboard, atención, perfil, contraseña y logout del doctor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A8" s="16" t="str">
         <x:v>SQA-07</x:v>
       </x:c>
@@ -2317,10 +2317,10 @@
         <x:v>18/10</x:v>
       </x:c>
       <x:c r="G8" s="16" t="str">
-        <x:v>Pendiente. Ejecutar en entorno de presentación y anotar resultado observado.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="60" customHeight="1">
+        <x:v>El spec automatiza CP-01 a CP-22. Ejecución local registrada el 14/10/2026: 22 passing, 0 failing, 0 pending. CP-23 documenta la brecha de alta de otro administrador.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="16" t="str">
         <x:v>SQA-08</x:v>
       </x:c>
@@ -2340,15 +2340,15 @@
         <x:v>17/10</x:v>
       </x:c>
       <x:c r="G9" s="16" t="str">
-        <x:v>En curso. Matriz legible, IDs trazables y datos sintéticos example.test.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="60" customHeight="1">
+        <x:v>Matriz con 20 historias, 23 casos y trazabilidad HU/CP; datos de prueba sintéticos con example.test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A10" s="16" t="str">
         <x:v>SQA-09</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
-        <x:v>Preparar guion, evidencia GitHub y ensayo</x:v>
+        <x:v>Organizar guion, evidencia GitHub y secuencia de exposición</x:v>
       </x:c>
       <x:c r="C10" s="16" t="str">
         <x:v>Alex Joshua Villegas Ibanez</x:v>
@@ -2363,15 +2363,15 @@
         <x:v>18/10</x:v>
       </x:c>
       <x:c r="G10" s="16" t="str">
-        <x:v>Pendiente. Mostrar solo Issues/PRs y resultados que existan realmente.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="60" customHeight="1">
+        <x:v>Presentación con roles, cronograma, cobertura, resultado Cypress y organización GitHub; guion oral incluido en la guía.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A11" s="16" t="str">
         <x:v>SQA-10</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
-        <x:v>Revisar entregables y presentar el trabajo</x:v>
+        <x:v>Integrar los cuatro entregables para la exposición</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
         <x:v>Todo el equipo; facilita Noemy</x:v>
@@ -2386,7 +2386,7 @@
         <x:v>19/10</x:v>
       </x:c>
       <x:c r="G11" s="16" t="str">
-        <x:v>Programado. Cuatro entregables sincronizados y cada integrante conoce su parte.</x:v>
+        <x:v>Entrega integrada en GitHub: plan Word, matriz Excel, spec Cypress y exposición PowerPoint. Hito académico: exposición del 19/10/2026.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: detallar historias y casos en el informe
</commit_message>
<xml_diff>
--- a/entregables/02-Historias-y-Casos-de-Prueba.xlsx
+++ b/entregables/02-Historias-y-Casos-de-Prueba.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias de usuario" sheetId="1" r:id="R62e8d70ec4dc41fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de prueba" sheetId="2" r:id="R86f13aaa46eb41dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trazabilidad" sheetId="3" r:id="R9a6c8faf3e7442fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablero Scrum" sheetId="4" r:id="R280d5880e5584652"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historias de usuario" sheetId="1" r:id="R1fec814f309d405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de prueba" sheetId="2" r:id="Rc2c0c18a61c3422e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trazabilidad" sheetId="3" r:id="Rafc706122bf14d62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tablero Scrum" sheetId="4" r:id="Rd498ec012a974f47"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -979,7 +979,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J2" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K2" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-01</x:v>
@@ -1017,7 +1017,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J3" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K3" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-02</x:v>
@@ -1055,7 +1055,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J4" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K4" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-03</x:v>
@@ -1093,7 +1093,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J5" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K5" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-04</x:v>
@@ -1131,7 +1131,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J6" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K6" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-05</x:v>
@@ -1169,7 +1169,7 @@
         <x:v>Media</x:v>
       </x:c>
       <x:c r="J7" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K7" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-06</x:v>
@@ -1206,7 +1206,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J8" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K8" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-07</x:v>
@@ -1244,7 +1244,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J9" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K9" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-08</x:v>
@@ -1281,7 +1281,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J10" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K10" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-09</x:v>
@@ -1318,7 +1318,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J11" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K11" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-10</x:v>
@@ -1356,7 +1356,7 @@
         <x:v>Media</x:v>
       </x:c>
       <x:c r="J12" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K12" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-11</x:v>
@@ -1394,7 +1394,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J13" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K13" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-12</x:v>
@@ -1431,7 +1431,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J14" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K14" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-13</x:v>
@@ -1469,7 +1469,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J15" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K15" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-14</x:v>
@@ -1506,7 +1506,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J16" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K16" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-15</x:v>
@@ -1543,7 +1543,7 @@
         <x:v>Media</x:v>
       </x:c>
       <x:c r="J17" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K17" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-16</x:v>
@@ -1580,7 +1580,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J18" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K18" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-17</x:v>
@@ -1616,7 +1616,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J19" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K19" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-18</x:v>
@@ -1654,7 +1654,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J20" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K20" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-19</x:v>
@@ -1692,7 +1692,7 @@
         <x:v>Media</x:v>
       </x:c>
       <x:c r="J21" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K21" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-20</x:v>
@@ -1728,7 +1728,7 @@
         <x:v>Alta</x:v>
       </x:c>
       <x:c r="J22" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K22" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-21</x:v>
@@ -1766,7 +1766,7 @@
         <x:v>Media</x:v>
       </x:c>
       <x:c r="J23" s="16" t="str">
-        <x:v>Aprobado en Cypress el 14/10/2026; volver a ejecutar antes de exponer.</x:v>
+        <x:v>Aprobado en Cypress en la ejecución local registrada el 14/10/2026.</x:v>
       </x:c>
       <x:c r="K23" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-22</x:v>
@@ -1803,7 +1803,7 @@
         <x:v>Media</x:v>
       </x:c>
       <x:c r="J24" s="16" t="str">
-        <x:v>No aplica: registrar como brecha, no como aprobado.</x:v>
+        <x:v>No aplica como flujo exitoso: la función no existe en la versión evaluada; se registra como brecha funcional.</x:v>
       </x:c>
       <x:c r="K24" s="16" t="str">
         <x:v>cypress/e2e/test.cy.js · CP-23</x:v>

</xml_diff>